<commit_message>
refactor: update data directory management for environment compatibility
</commit_message>
<xml_diff>
--- a/data/對照表.xlsx
+++ b/data/對照表.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,249 +455,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>[夏天必備☀️打底神器]內搭襯裙 背帶裙 細肩帶睡衣 長版背心::【黑色】吊帶款▶短版,L</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>蝦皮</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>M型短頸膚感防滑衣架[奶霧灰]</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>HGI03023-GY</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>HGI03023</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>[高回購口碑款🍑超好穿不夾臀] 高腰內褲 女生內褲 莫代爾 女內著 內褲女::煙粉色,M</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>蝦皮</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>M型短頸膚感防滑衣架[黑色]</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>HGI03023-BK</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>HGI03023</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>123::123::123</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>露天</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>M型短頸膚感防滑衣架[燕麥白]</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>HGI03023-WH</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>HGI03023</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>[台灣冠軍🏆爆賣30萬件]冰絲內褲 男內褲 涼感內褲 男士內褲 平口褲::寶藍色::L ➜建議70-75KG</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>露天</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>厚磅撞色圓領短版修身短袖T恤[深藍M]</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>HFA01019-DN-M</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>HFA01019</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>[台灣冠軍🏆爆賣30萬件]冰絲內褲 男內褲 涼感內褲 男士內褲 平口褲::白色::XL ➜建議80-85KG</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>露天</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>厚磅撞色圓領短版修身短袖T恤[深藍XL]</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>HFA01019-DN-XL</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>HFA01019</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>新品限時優惠❇️秋冬萬用打底衣🍁柔軟高彈莫代爾內搭長袖上衣｜長袖T恤 圓領上衣 高領 翻領 長T 內搭衣 長袖TEE::白色｜高領::L</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>露天</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>厚磅撞色圓領短版修身短袖T恤[杏色XL]</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>HFA01019-BG-XL</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>HFA01019</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>真好穿🌷不捲邊不夾臀🍑裸感60S莫代爾超舒適加寬邊中高腰內褲三角褲::米咖色, M</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>官網</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>厚磅撞色圓領短版修身短袖T恤[深藍XL]</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>HFA01019-DN-XL</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>HFA01019</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>超柔順莫代爾棉☁️高質感彩紗條紋男性四角內褲::【素色】黑灰色, XL ➜建議80-85KG</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>官網</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>厚磅撞色圓領短版修身短袖T恤[深藍XL]</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>HFA01019-DN-XL</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>HFA01019</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>超輕薄涼爽無痕零觸感！高品質舒適彈力冰絲四角內褲::黑色, L ➜建議70-75KG</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>官網</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>厚磅撞色圓領短版修身短袖T恤[深藍M]</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>HFA01019-DN-M</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>HFA01019</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>